<commit_message>
Enrichir l'expertise de Romain Rissoan (LinkedIn + sites experts IA)
Description détaillée intégrant son profil LinkedIn et les expertises
présentées sur expert-ia-assurance-banque.fr, expert-ia-medico-social.fr,
expert-claude-ai.fr et conferencier-expert-ia.fr : parcours, secteurs,
prestations (conseil, agents IA, formation Qualiopi, conformité,
conférences), technologies et chiffres clés. Synchronisé CSV/JSON/XLSX.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Les-Experts-en-Intelligence-Artificielle.xlsx
+++ b/Les-Experts-en-Intelligence-Artificielle.xlsx
@@ -49,7 +49,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -60,6 +60,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,7 +392,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>Professeur en informatique théorique à l'ENS Lyon, spécialiste de la complexité algorithmique</t>
         </is>
@@ -416,7 +419,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>Chercheur en vision par ordinateur et apprentissage profond appliqués à la robotique</t>
         </is>
@@ -443,7 +446,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>Chercheur en IA développementale et robotique constructiviste à l'UCLy</t>
         </is>
@@ -470,9 +473,9 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Consultant-formateur en IA générative (GPT, LLM), fondateur d'Opcadia à Lyon</t>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Fondateur d'Opcadia (Lyon) et de la marque Expert IA Assurance Banque ; consultant-formateur digital depuis 2009, projets d'IA prédictive (scoring, détection de fraude, automatisation des processus) depuis 2015 et IA générative depuis 2023. Accompagne banques, assureurs, finance et secteur médico-social sur tout le cycle de vie des projets IA : cadrage stratégique en comité exécutif, prototypage rapide, intégration système (API Claude, Claude Agent SDK, Model Context Protocol, Claude Code), mise en production et conformité AI Act / RGPD. Développement d'agents IA et d'assistants métier (service client, automatisation documentaire, assistants juridiques, solutions finance/assurance). Formateur certifié Qualiopi (ChatGPT, Claude, Mistral, Midjourney, Copilot, Heygen ; ingénierie de prompts), plus de 10 000 personnes formées et ~100 jours de conférences et keynotes par an. Auteur de 5 ouvrages dont 2 sur l'IA, 20 000 abonnés LinkedIn, bilingue anglais (France, Belgique, Luxembourg, Suisse).</t>
         </is>
       </c>
     </row>
@@ -497,7 +500,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>Consultant-formateur en marketing digital, IA et stratégie sur les réseaux sociaux</t>
         </is>
@@ -524,7 +527,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>Cofondateur et CEO de Mistral AI, spécialiste des grands modèles de langage (LLM)</t>
         </is>
@@ -551,7 +554,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>Cofondateur et CEO de Hugging Face, figure de l'IA open source et du machine learning</t>
         </is>
@@ -578,7 +581,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>Directrice de l'institut PRAIRIE, experte en IA et politiques d'innovation</t>
         </is>
@@ -605,7 +608,7 @@
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>Directeur de recherche Inria, IA développementale et apprentissage par curiosité chez les robots</t>
         </is>
@@ -632,7 +635,7 @@
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>Professeur en recherche opérationnelle, optimisation combinatoire et programmation mathématique</t>
         </is>
@@ -659,7 +662,7 @@
           <t>Marseille</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>Spécialiste du machine learning : méthodes à noyaux et apprentissage statistique</t>
         </is>
@@ -686,7 +689,7 @@
           <t>Marseille</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'IA symbolique et du diagnostic de systèmes à base de modèles</t>
         </is>
@@ -713,7 +716,7 @@
           <t>Nantes</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>Professeur en modèles graphiques probabilistes, réseaux bayésiens et découverte causale</t>
         </is>
@@ -740,7 +743,7 @@
           <t>Nantes</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>Chercheur en traitement automatique des langues et fouille de textes par motifs</t>
         </is>
@@ -767,7 +770,7 @@
           <t>Rennes</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>Chercheur Inria en asservissement visuel et robotique fondée sur la vision</t>
         </is>
@@ -794,7 +797,7 @@
           <t>Rennes</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>Chercheur Meta AI, créateur de FAISS, recherche de similarité vectorielle à grande échelle</t>
         </is>
@@ -821,7 +824,7 @@
           <t>Lille</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>Pionnier de l'apprentissage automatique et de l'apprentissage par renforcement séquentiel</t>
         </is>
@@ -848,7 +851,7 @@
           <t>Lille</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>Expert en vision par ordinateur, apprentissage profond et indexation d'images</t>
         </is>
@@ -875,7 +878,7 @@
           <t>Grenoble</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'apprentissage automatique, de l'optimisation et de la vision par ordinateur</t>
         </is>
@@ -902,7 +905,7 @@
           <t>Grenoble</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'apprentissage multimodal audio-visuel pour l'interaction homme-robot</t>
         </is>
@@ -929,7 +932,7 @@
           <t>Grenoble</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>Chercheuse de renommée mondiale en vision par ordinateur et apprentissage profond</t>
         </is>
@@ -956,7 +959,7 @@
           <t>Clermont-Ferrand</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de la fouille de données, extraction de motifs et analyse formelle de concepts</t>
         </is>
@@ -983,7 +986,7 @@
           <t>Clermont-Ferrand</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'apprentissage symbolique, programmation logique inductive et fouille de données</t>
         </is>
@@ -1010,7 +1013,7 @@
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de la vision par ordinateur appliquée à l'analyse des activités chirurgicales</t>
         </is>
@@ -1037,7 +1040,7 @@
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>Chercheur en intelligence artificielle et apprentissage automatique (laboratoire ICube, Strasbourg)</t>
         </is>
@@ -1064,7 +1067,7 @@
           <t>Metz</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'IA responsable, des systèmes compagnons intelligents et de l'e-éducation</t>
         </is>
@@ -1091,7 +1094,7 @@
           <t>Metz</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>Chercheur en informatique et intelligence artificielle (Université de Lorraine, Metz)</t>
         </is>
@@ -1118,7 +1121,7 @@
           <t>Caen</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de la vision par ordinateur et de l'apprentissage profond pour la reconnaissance d'objets</t>
         </is>
@@ -1145,7 +1148,7 @@
           <t>Caen</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>Spécialiste du traitement du signal audio, de la parole et de la reconnaissance du locuteur</t>
         </is>
@@ -1172,7 +1175,7 @@
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de la sémantique formelle, de la pragmatique du discours et du TAL</t>
         </is>
@@ -1199,7 +1202,7 @@
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>Spécialiste du traitement du signal et de l'imagerie hyperspectrale par méthodes bayésiennes</t>
         </is>
@@ -1226,7 +1229,7 @@
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de la robotique et de la programmation bayésienne pour la perception et l'action</t>
         </is>
@@ -1253,7 +1256,7 @@
           <t>Nice</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>Directeur de recherche Inria, IA pour l'imagerie médicale et le patient numérique</t>
         </is>
@@ -1280,7 +1283,7 @@
           <t>Nice</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>Professeur de statistique, apprentissage statistique en grande dimension et données complexes</t>
         </is>
@@ -1307,7 +1310,7 @@
           <t>Nice</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>Professeur d'informatique, apprentissage automatique et réseaux de neurones sous contraintes</t>
         </is>
@@ -1334,7 +1337,7 @@
           <t>Pau</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>Professeur, IA et apprentissage pour systèmes cyber-physiques et IoT (Industrie 4.0)</t>
         </is>
@@ -1361,7 +1364,7 @@
           <t>Pau</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>Professeur de mathématiques, statistiques, quantification d'incertitude et analyse de sensibilité</t>
         </is>
@@ -1388,7 +1391,7 @@
           <t>Tours</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>Chercheur en TAL, automates et transducteurs pour la reconnaissance d'entités nommées</t>
         </is>
@@ -1415,7 +1418,7 @@
           <t>Tours</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>Professeur, fouille de données et extraction de motifs fréquents à grande échelle</t>
         </is>
@@ -1442,7 +1445,7 @@
           <t>Orléans</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>Spécialiste de l'apprentissage symbolique, programmation logique inductive et fouille de données</t>
         </is>
@@ -1469,7 +1472,7 @@
           <t>Orléans</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>Chercheuse en représentation des connaissances et fouille de données spatio-temporelles</t>
         </is>

</xml_diff>